<commit_message>
📊 Update reports — Build #6
</commit_message>
<xml_diff>
--- a/reports/appium/Excel/Automation_Test_Report.xlsx
+++ b/reports/appium/Excel/Automation_Test_Report.xlsx
@@ -502,7 +502,7 @@
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Build #1  |  2026-06-23 07:39 UTC  |  Total: 0  |  Passed: 0  |  Failed: 0</t>
+          <t>Build #6  |  2026-06-23 08:20 UTC  |  Total: 0  |  Passed: 0  |  Failed: 0</t>
         </is>
       </c>
     </row>
@@ -736,7 +736,7 @@
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>#1</t>
+          <t>#6</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr"/>

</xml_diff>

<commit_message>
📊 Update reports — Build #11
</commit_message>
<xml_diff>
--- a/reports/appium/Excel/Automation_Test_Report.xlsx
+++ b/reports/appium/Excel/Automation_Test_Report.xlsx
@@ -1247,13 +1247,13 @@
     <t>Build Number</t>
   </si>
   <si>
-    <t>10</t>
+    <t>11</t>
   </si>
   <si>
     <t>Execution Date</t>
   </si>
   <si>
-    <t>2026-06-23 11:22:27 UTC</t>
+    <t>2026-06-23 12:04:54 UTC</t>
   </si>
   <si>
     <t>Branch</t>
@@ -1265,7 +1265,7 @@
     <t>Commit</t>
   </si>
   <si>
-    <t>edcce0c</t>
+    <t>348580a</t>
   </si>
   <si>
     <t>Total</t>

</xml_diff>

<commit_message>
📊 Update reports — Build #12
</commit_message>
<xml_diff>
--- a/reports/appium/Excel/Automation_Test_Report.xlsx
+++ b/reports/appium/Excel/Automation_Test_Report.xlsx
@@ -1247,13 +1247,13 @@
     <t>Build Number</t>
   </si>
   <si>
-    <t>11</t>
+    <t>12</t>
   </si>
   <si>
     <t>Execution Date</t>
   </si>
   <si>
-    <t>2026-06-23 12:04:54 UTC</t>
+    <t>2026-06-23 13:17:31 UTC</t>
   </si>
   <si>
     <t>Branch</t>
@@ -1265,7 +1265,7 @@
     <t>Commit</t>
   </si>
   <si>
-    <t>348580a</t>
+    <t>cfbb4d3</t>
   </si>
   <si>
     <t>Total</t>

</xml_diff>

<commit_message>
📊 Update reports — Build #14
</commit_message>
<xml_diff>
--- a/reports/appium/Excel/Automation_Test_Report.xlsx
+++ b/reports/appium/Excel/Automation_Test_Report.xlsx
@@ -1247,13 +1247,13 @@
     <t>Build Number</t>
   </si>
   <si>
-    <t>12</t>
+    <t>14</t>
   </si>
   <si>
     <t>Execution Date</t>
   </si>
   <si>
-    <t>2026-06-23 13:17:31 UTC</t>
+    <t>2026-06-23 13:38:15 UTC</t>
   </si>
   <si>
     <t>Branch</t>
@@ -1265,7 +1265,7 @@
     <t>Commit</t>
   </si>
   <si>
-    <t>cfbb4d3</t>
+    <t>3eb8262</t>
   </si>
   <si>
     <t>Total</t>

</xml_diff>

<commit_message>
📊 Update reports — Build #15
</commit_message>
<xml_diff>
--- a/reports/appium/Excel/Automation_Test_Report.xlsx
+++ b/reports/appium/Excel/Automation_Test_Report.xlsx
@@ -1247,13 +1247,13 @@
     <t>Build Number</t>
   </si>
   <si>
-    <t>14</t>
+    <t>15</t>
   </si>
   <si>
     <t>Execution Date</t>
   </si>
   <si>
-    <t>2026-06-23 13:38:15 UTC</t>
+    <t>2026-06-23 13:48:10 UTC</t>
   </si>
   <si>
     <t>Branch</t>
@@ -1265,7 +1265,7 @@
     <t>Commit</t>
   </si>
   <si>
-    <t>3eb8262</t>
+    <t>0bdfd4b</t>
   </si>
   <si>
     <t>Total</t>

</xml_diff>

<commit_message>
📊 Update reports — Build #16
</commit_message>
<xml_diff>
--- a/reports/appium/Excel/Automation_Test_Report.xlsx
+++ b/reports/appium/Excel/Automation_Test_Report.xlsx
@@ -1247,13 +1247,13 @@
     <t>Build Number</t>
   </si>
   <si>
-    <t>15</t>
+    <t>16</t>
   </si>
   <si>
     <t>Execution Date</t>
   </si>
   <si>
-    <t>2026-06-23 13:48:10 UTC</t>
+    <t>2026-06-23 13:56:35 UTC</t>
   </si>
   <si>
     <t>Branch</t>
@@ -1265,7 +1265,7 @@
     <t>Commit</t>
   </si>
   <si>
-    <t>0bdfd4b</t>
+    <t>e40a5d4</t>
   </si>
   <si>
     <t>Total</t>

</xml_diff>

<commit_message>
📊 Update reports — Build #17
</commit_message>
<xml_diff>
--- a/reports/appium/Excel/Automation_Test_Report.xlsx
+++ b/reports/appium/Excel/Automation_Test_Report.xlsx
@@ -1247,13 +1247,13 @@
     <t>Build Number</t>
   </si>
   <si>
-    <t>16</t>
+    <t>17</t>
   </si>
   <si>
     <t>Execution Date</t>
   </si>
   <si>
-    <t>2026-06-23 13:56:35 UTC</t>
+    <t>2026-06-23 14:23:37 UTC</t>
   </si>
   <si>
     <t>Branch</t>
@@ -1265,7 +1265,7 @@
     <t>Commit</t>
   </si>
   <si>
-    <t>e40a5d4</t>
+    <t>d1d53d0</t>
   </si>
   <si>
     <t>Total</t>

</xml_diff>

<commit_message>
📊 Update reports — Build #18
</commit_message>
<xml_diff>
--- a/reports/appium/Excel/Automation_Test_Report.xlsx
+++ b/reports/appium/Excel/Automation_Test_Report.xlsx
@@ -1247,13 +1247,13 @@
     <t>Build Number</t>
   </si>
   <si>
-    <t>17</t>
+    <t>18</t>
   </si>
   <si>
     <t>Execution Date</t>
   </si>
   <si>
-    <t>2026-06-23 14:23:37 UTC</t>
+    <t>2026-06-23 14:33:32 UTC</t>
   </si>
   <si>
     <t>Branch</t>
@@ -1265,7 +1265,7 @@
     <t>Commit</t>
   </si>
   <si>
-    <t>d1d53d0</t>
+    <t>04fd2d2</t>
   </si>
   <si>
     <t>Total</t>

</xml_diff>

<commit_message>
📊 Update reports — Build #19
</commit_message>
<xml_diff>
--- a/reports/appium/Excel/Automation_Test_Report.xlsx
+++ b/reports/appium/Excel/Automation_Test_Report.xlsx
@@ -1247,13 +1247,13 @@
     <t>Build Number</t>
   </si>
   <si>
-    <t>18</t>
+    <t>19</t>
   </si>
   <si>
     <t>Execution Date</t>
   </si>
   <si>
-    <t>2026-06-23 14:33:32 UTC</t>
+    <t>2026-06-23 14:55:04 UTC</t>
   </si>
   <si>
     <t>Branch</t>
@@ -1265,7 +1265,7 @@
     <t>Commit</t>
   </si>
   <si>
-    <t>04fd2d2</t>
+    <t>af530d5</t>
   </si>
   <si>
     <t>Total</t>

</xml_diff>

<commit_message>
📊 Update reports — Build #20
</commit_message>
<xml_diff>
--- a/reports/appium/Excel/Automation_Test_Report.xlsx
+++ b/reports/appium/Excel/Automation_Test_Report.xlsx
@@ -1247,13 +1247,13 @@
     <t>Build Number</t>
   </si>
   <si>
-    <t>19</t>
+    <t>20</t>
   </si>
   <si>
     <t>Execution Date</t>
   </si>
   <si>
-    <t>2026-06-23 14:55:04 UTC</t>
+    <t>2026-06-23 15:16:29 UTC</t>
   </si>
   <si>
     <t>Branch</t>
@@ -1265,7 +1265,7 @@
     <t>Commit</t>
   </si>
   <si>
-    <t>af530d5</t>
+    <t>a38f0ce</t>
   </si>
   <si>
     <t>Total</t>

</xml_diff>

<commit_message>
📊 Update reports — Build #21
</commit_message>
<xml_diff>
--- a/reports/appium/Excel/Automation_Test_Report.xlsx
+++ b/reports/appium/Excel/Automation_Test_Report.xlsx
@@ -1247,13 +1247,13 @@
     <t>Build Number</t>
   </si>
   <si>
-    <t>20</t>
+    <t>21</t>
   </si>
   <si>
     <t>Execution Date</t>
   </si>
   <si>
-    <t>2026-06-23 15:16:29 UTC</t>
+    <t>2026-06-23 15:20:13 UTC</t>
   </si>
   <si>
     <t>Branch</t>
@@ -1265,7 +1265,7 @@
     <t>Commit</t>
   </si>
   <si>
-    <t>a38f0ce</t>
+    <t>6a5e7ca</t>
   </si>
   <si>
     <t>Total</t>

</xml_diff>

<commit_message>
📊 Update reports — Build #22
</commit_message>
<xml_diff>
--- a/reports/appium/Excel/Automation_Test_Report.xlsx
+++ b/reports/appium/Excel/Automation_Test_Report.xlsx
@@ -1247,13 +1247,13 @@
     <t>Build Number</t>
   </si>
   <si>
-    <t>21</t>
+    <t>22</t>
   </si>
   <si>
     <t>Execution Date</t>
   </si>
   <si>
-    <t>2026-06-23 15:20:13 UTC</t>
+    <t>2026-06-23 15:33:09 UTC</t>
   </si>
   <si>
     <t>Branch</t>
@@ -1265,7 +1265,7 @@
     <t>Commit</t>
   </si>
   <si>
-    <t>6a5e7ca</t>
+    <t>f8042b0</t>
   </si>
   <si>
     <t>Total</t>

</xml_diff>

<commit_message>
📊 Update reports — Build #23
</commit_message>
<xml_diff>
--- a/reports/appium/Excel/Automation_Test_Report.xlsx
+++ b/reports/appium/Excel/Automation_Test_Report.xlsx
@@ -1247,13 +1247,13 @@
     <t>Build Number</t>
   </si>
   <si>
-    <t>22</t>
+    <t>23</t>
   </si>
   <si>
     <t>Execution Date</t>
   </si>
   <si>
-    <t>2026-06-23 15:33:09 UTC</t>
+    <t>2026-06-23 15:39:57 UTC</t>
   </si>
   <si>
     <t>Branch</t>
@@ -1265,7 +1265,7 @@
     <t>Commit</t>
   </si>
   <si>
-    <t>f8042b0</t>
+    <t>19701a0</t>
   </si>
   <si>
     <t>Total</t>

</xml_diff>

<commit_message>
📊 Update reports — Build #24
</commit_message>
<xml_diff>
--- a/reports/appium/Excel/Automation_Test_Report.xlsx
+++ b/reports/appium/Excel/Automation_Test_Report.xlsx
@@ -1247,13 +1247,13 @@
     <t>Build Number</t>
   </si>
   <si>
-    <t>23</t>
+    <t>24</t>
   </si>
   <si>
     <t>Execution Date</t>
   </si>
   <si>
-    <t>2026-06-23 15:39:57 UTC</t>
+    <t>2026-06-24 03:32:59 UTC</t>
   </si>
   <si>
     <t>Branch</t>

</xml_diff>

<commit_message>
📊 Update reports — Build #25
</commit_message>
<xml_diff>
--- a/reports/appium/Excel/Automation_Test_Report.xlsx
+++ b/reports/appium/Excel/Automation_Test_Report.xlsx
@@ -1247,13 +1247,13 @@
     <t>Build Number</t>
   </si>
   <si>
-    <t>24</t>
+    <t>25</t>
   </si>
   <si>
     <t>Execution Date</t>
   </si>
   <si>
-    <t>2026-06-24 03:32:59 UTC</t>
+    <t>2026-06-24 04:39:26 UTC</t>
   </si>
   <si>
     <t>Branch</t>
@@ -1265,7 +1265,7 @@
     <t>Commit</t>
   </si>
   <si>
-    <t>19701a0</t>
+    <t>f6dc91b</t>
   </si>
   <si>
     <t>Total</t>

</xml_diff>

<commit_message>
📊 Update reports — Build #26
</commit_message>
<xml_diff>
--- a/reports/appium/Excel/Automation_Test_Report.xlsx
+++ b/reports/appium/Excel/Automation_Test_Report.xlsx
@@ -1247,13 +1247,13 @@
     <t>Build Number</t>
   </si>
   <si>
-    <t>25</t>
+    <t>26</t>
   </si>
   <si>
     <t>Execution Date</t>
   </si>
   <si>
-    <t>2026-06-24 04:39:26 UTC</t>
+    <t>2026-06-30 08:35:35 UTC</t>
   </si>
   <si>
     <t>Branch</t>
@@ -1265,7 +1265,7 @@
     <t>Commit</t>
   </si>
   <si>
-    <t>f6dc91b</t>
+    <t>1b19601</t>
   </si>
   <si>
     <t>Total</t>

</xml_diff>

<commit_message>
📊 Update reports — Build #27
</commit_message>
<xml_diff>
--- a/reports/appium/Excel/Automation_Test_Report.xlsx
+++ b/reports/appium/Excel/Automation_Test_Report.xlsx
@@ -1247,13 +1247,13 @@
     <t>Build Number</t>
   </si>
   <si>
-    <t>26</t>
+    <t>27</t>
   </si>
   <si>
     <t>Execution Date</t>
   </si>
   <si>
-    <t>2026-06-30 08:35:35 UTC</t>
+    <t>2026-06-30 13:20:01 UTC</t>
   </si>
   <si>
     <t>Branch</t>
@@ -1265,7 +1265,7 @@
     <t>Commit</t>
   </si>
   <si>
-    <t>1b19601</t>
+    <t>9a48722</t>
   </si>
   <si>
     <t>Total</t>

</xml_diff>

<commit_message>
📊 Update reports — Build #28
</commit_message>
<xml_diff>
--- a/reports/appium/Excel/Automation_Test_Report.xlsx
+++ b/reports/appium/Excel/Automation_Test_Report.xlsx
@@ -1247,13 +1247,13 @@
     <t>Build Number</t>
   </si>
   <si>
-    <t>27</t>
+    <t>28</t>
   </si>
   <si>
     <t>Execution Date</t>
   </si>
   <si>
-    <t>2026-06-30 13:20:01 UTC</t>
+    <t>2026-06-30 13:28:08 UTC</t>
   </si>
   <si>
     <t>Branch</t>
@@ -1265,7 +1265,7 @@
     <t>Commit</t>
   </si>
   <si>
-    <t>9a48722</t>
+    <t>7bb6a7a</t>
   </si>
   <si>
     <t>Total</t>

</xml_diff>

<commit_message>
📊 Update reports — Build #29
</commit_message>
<xml_diff>
--- a/reports/appium/Excel/Automation_Test_Report.xlsx
+++ b/reports/appium/Excel/Automation_Test_Report.xlsx
@@ -1247,13 +1247,13 @@
     <t>Build Number</t>
   </si>
   <si>
-    <t>28</t>
+    <t>29</t>
   </si>
   <si>
     <t>Execution Date</t>
   </si>
   <si>
-    <t>2026-06-30 13:28:08 UTC</t>
+    <t>2026-06-30 13:37:06 UTC</t>
   </si>
   <si>
     <t>Branch</t>
@@ -1265,7 +1265,7 @@
     <t>Commit</t>
   </si>
   <si>
-    <t>7bb6a7a</t>
+    <t>c744b19</t>
   </si>
   <si>
     <t>Total</t>

</xml_diff>

<commit_message>
📊 Update reports — Build #30
</commit_message>
<xml_diff>
--- a/reports/appium/Excel/Automation_Test_Report.xlsx
+++ b/reports/appium/Excel/Automation_Test_Report.xlsx
@@ -1247,13 +1247,13 @@
     <t>Build Number</t>
   </si>
   <si>
-    <t>29</t>
+    <t>30</t>
   </si>
   <si>
     <t>Execution Date</t>
   </si>
   <si>
-    <t>2026-06-30 13:37:06 UTC</t>
+    <t>2026-06-30 13:44:53 UTC</t>
   </si>
   <si>
     <t>Branch</t>
@@ -1265,7 +1265,7 @@
     <t>Commit</t>
   </si>
   <si>
-    <t>c744b19</t>
+    <t>6c162b2</t>
   </si>
   <si>
     <t>Total</t>

</xml_diff>

<commit_message>
📊 Update reports — Build #31
</commit_message>
<xml_diff>
--- a/reports/appium/Excel/Automation_Test_Report.xlsx
+++ b/reports/appium/Excel/Automation_Test_Report.xlsx
@@ -1247,13 +1247,13 @@
     <t>Build Number</t>
   </si>
   <si>
-    <t>30</t>
+    <t>31</t>
   </si>
   <si>
     <t>Execution Date</t>
   </si>
   <si>
-    <t>2026-06-30 13:44:53 UTC</t>
+    <t>2026-06-30 13:52:56 UTC</t>
   </si>
   <si>
     <t>Branch</t>
@@ -1265,7 +1265,7 @@
     <t>Commit</t>
   </si>
   <si>
-    <t>6c162b2</t>
+    <t>4e802ad</t>
   </si>
   <si>
     <t>Total</t>

</xml_diff>

<commit_message>
📊 Update reports — Build #32
</commit_message>
<xml_diff>
--- a/reports/appium/Excel/Automation_Test_Report.xlsx
+++ b/reports/appium/Excel/Automation_Test_Report.xlsx
@@ -1247,13 +1247,13 @@
     <t>Build Number</t>
   </si>
   <si>
-    <t>31</t>
+    <t>32</t>
   </si>
   <si>
     <t>Execution Date</t>
   </si>
   <si>
-    <t>2026-06-30 13:52:56 UTC</t>
+    <t>2026-06-30 14:15:50 UTC</t>
   </si>
   <si>
     <t>Branch</t>
@@ -1265,7 +1265,7 @@
     <t>Commit</t>
   </si>
   <si>
-    <t>4e802ad</t>
+    <t>36ef16e</t>
   </si>
   <si>
     <t>Total</t>

</xml_diff>

<commit_message>
📊 Update reports — Build #34
</commit_message>
<xml_diff>
--- a/reports/appium/Excel/Automation_Test_Report.xlsx
+++ b/reports/appium/Excel/Automation_Test_Report.xlsx
@@ -1247,13 +1247,13 @@
     <t>Build Number</t>
   </si>
   <si>
-    <t>32</t>
+    <t>34</t>
   </si>
   <si>
     <t>Execution Date</t>
   </si>
   <si>
-    <t>2026-06-30 14:15:50 UTC</t>
+    <t>2026-06-30 14:26:49 UTC</t>
   </si>
   <si>
     <t>Branch</t>
@@ -1265,7 +1265,7 @@
     <t>Commit</t>
   </si>
   <si>
-    <t>36ef16e</t>
+    <t>16d388e</t>
   </si>
   <si>
     <t>Total</t>

</xml_diff>

<commit_message>
📊 Update reports — Build #36
</commit_message>
<xml_diff>
--- a/reports/appium/Excel/Automation_Test_Report.xlsx
+++ b/reports/appium/Excel/Automation_Test_Report.xlsx
@@ -1247,13 +1247,13 @@
     <t>Build Number</t>
   </si>
   <si>
-    <t>34</t>
+    <t>36</t>
   </si>
   <si>
     <t>Execution Date</t>
   </si>
   <si>
-    <t>2026-06-30 14:26:49 UTC</t>
+    <t>2026-06-30 14:33:32 UTC</t>
   </si>
   <si>
     <t>Branch</t>
@@ -1265,7 +1265,7 @@
     <t>Commit</t>
   </si>
   <si>
-    <t>16d388e</t>
+    <t>c0c6499</t>
   </si>
   <si>
     <t>Total</t>

</xml_diff>

<commit_message>
📊 Update reports — Build #37
</commit_message>
<xml_diff>
--- a/reports/appium/Excel/Automation_Test_Report.xlsx
+++ b/reports/appium/Excel/Automation_Test_Report.xlsx
@@ -1247,13 +1247,13 @@
     <t>Build Number</t>
   </si>
   <si>
-    <t>36</t>
+    <t>37</t>
   </si>
   <si>
     <t>Execution Date</t>
   </si>
   <si>
-    <t>2026-06-30 14:33:32 UTC</t>
+    <t>2026-06-30 14:41:17 UTC</t>
   </si>
   <si>
     <t>Branch</t>
@@ -1265,7 +1265,7 @@
     <t>Commit</t>
   </si>
   <si>
-    <t>c0c6499</t>
+    <t>69c8bfb</t>
   </si>
   <si>
     <t>Total</t>

</xml_diff>

<commit_message>
📊 Update reports — Build #38
</commit_message>
<xml_diff>
--- a/reports/appium/Excel/Automation_Test_Report.xlsx
+++ b/reports/appium/Excel/Automation_Test_Report.xlsx
@@ -1247,13 +1247,13 @@
     <t>Build Number</t>
   </si>
   <si>
-    <t>37</t>
+    <t>38</t>
   </si>
   <si>
     <t>Execution Date</t>
   </si>
   <si>
-    <t>2026-06-30 14:41:17 UTC</t>
+    <t>2026-06-30 14:52:26 UTC</t>
   </si>
   <si>
     <t>Branch</t>
@@ -1265,7 +1265,7 @@
     <t>Commit</t>
   </si>
   <si>
-    <t>69c8bfb</t>
+    <t>8620bea</t>
   </si>
   <si>
     <t>Total</t>

</xml_diff>

<commit_message>
📊 Update reports — Build #39
</commit_message>
<xml_diff>
--- a/reports/appium/Excel/Automation_Test_Report.xlsx
+++ b/reports/appium/Excel/Automation_Test_Report.xlsx
@@ -1247,13 +1247,13 @@
     <t>Build Number</t>
   </si>
   <si>
-    <t>38</t>
+    <t>39</t>
   </si>
   <si>
     <t>Execution Date</t>
   </si>
   <si>
-    <t>2026-06-30 14:52:26 UTC</t>
+    <t>2026-06-30 15:10:34 UTC</t>
   </si>
   <si>
     <t>Branch</t>
@@ -1265,7 +1265,7 @@
     <t>Commit</t>
   </si>
   <si>
-    <t>8620bea</t>
+    <t>bbf0a04</t>
   </si>
   <si>
     <t>Total</t>

</xml_diff>

<commit_message>
📊 Update reports — Build #41
</commit_message>
<xml_diff>
--- a/reports/appium/Excel/Automation_Test_Report.xlsx
+++ b/reports/appium/Excel/Automation_Test_Report.xlsx
@@ -1247,13 +1247,13 @@
     <t>Build Number</t>
   </si>
   <si>
-    <t>39</t>
+    <t>41</t>
   </si>
   <si>
     <t>Execution Date</t>
   </si>
   <si>
-    <t>2026-06-30 15:10:34 UTC</t>
+    <t>2026-06-30 15:17:57 UTC</t>
   </si>
   <si>
     <t>Branch</t>
@@ -1265,7 +1265,7 @@
     <t>Commit</t>
   </si>
   <si>
-    <t>bbf0a04</t>
+    <t>2e22a52</t>
   </si>
   <si>
     <t>Total</t>

</xml_diff>

<commit_message>
📊 Update reports — Build #42
</commit_message>
<xml_diff>
--- a/reports/appium/Excel/Automation_Test_Report.xlsx
+++ b/reports/appium/Excel/Automation_Test_Report.xlsx
@@ -1247,13 +1247,13 @@
     <t>Build Number</t>
   </si>
   <si>
-    <t>41</t>
+    <t>42</t>
   </si>
   <si>
     <t>Execution Date</t>
   </si>
   <si>
-    <t>2026-06-30 15:17:57 UTC</t>
+    <t>2026-06-30 17:18:00 UTC</t>
   </si>
   <si>
     <t>Branch</t>
@@ -1265,7 +1265,7 @@
     <t>Commit</t>
   </si>
   <si>
-    <t>2e22a52</t>
+    <t>bb12b5d</t>
   </si>
   <si>
     <t>Total</t>

</xml_diff>

<commit_message>
📊 Update reports — Build #43
</commit_message>
<xml_diff>
--- a/reports/appium/Excel/Automation_Test_Report.xlsx
+++ b/reports/appium/Excel/Automation_Test_Report.xlsx
@@ -1247,13 +1247,13 @@
     <t>Build Number</t>
   </si>
   <si>
-    <t>42</t>
+    <t>43</t>
   </si>
   <si>
     <t>Execution Date</t>
   </si>
   <si>
-    <t>2026-06-30 17:18:00 UTC</t>
+    <t>2026-06-30 17:33:24 UTC</t>
   </si>
   <si>
     <t>Branch</t>
@@ -1265,7 +1265,7 @@
     <t>Commit</t>
   </si>
   <si>
-    <t>bb12b5d</t>
+    <t>feb30ad</t>
   </si>
   <si>
     <t>Total</t>

</xml_diff>

<commit_message>
📊 Update reports — Build #44
</commit_message>
<xml_diff>
--- a/reports/appium/Excel/Automation_Test_Report.xlsx
+++ b/reports/appium/Excel/Automation_Test_Report.xlsx
@@ -1247,13 +1247,13 @@
     <t>Build Number</t>
   </si>
   <si>
-    <t>43</t>
+    <t>44</t>
   </si>
   <si>
     <t>Execution Date</t>
   </si>
   <si>
-    <t>2026-06-30 17:33:24 UTC</t>
+    <t>2026-06-30 17:45:13 UTC</t>
   </si>
   <si>
     <t>Branch</t>
@@ -1265,7 +1265,7 @@
     <t>Commit</t>
   </si>
   <si>
-    <t>feb30ad</t>
+    <t>dfc30c0</t>
   </si>
   <si>
     <t>Total</t>

</xml_diff>

<commit_message>
📊 Update reports — Build #46
</commit_message>
<xml_diff>
--- a/reports/appium/Excel/Automation_Test_Report.xlsx
+++ b/reports/appium/Excel/Automation_Test_Report.xlsx
@@ -1247,13 +1247,13 @@
     <t>Build Number</t>
   </si>
   <si>
-    <t>45</t>
+    <t>46</t>
   </si>
   <si>
     <t>Execution Date</t>
   </si>
   <si>
-    <t>2026-07-20 04:26:42 UTC</t>
+    <t>2026-07-20 04:48:09 UTC</t>
   </si>
   <si>
     <t>Branch</t>
@@ -1265,7 +1265,7 @@
     <t>Commit</t>
   </si>
   <si>
-    <t>6c3e421</t>
+    <t>f5c0ab7</t>
   </si>
   <si>
     <t>Total</t>

</xml_diff>

<commit_message>
📊 Update reports — Build #47
</commit_message>
<xml_diff>
--- a/reports/appium/Excel/Automation_Test_Report.xlsx
+++ b/reports/appium/Excel/Automation_Test_Report.xlsx
@@ -1247,13 +1247,13 @@
     <t>Build Number</t>
   </si>
   <si>
-    <t>46</t>
+    <t>47</t>
   </si>
   <si>
     <t>Execution Date</t>
   </si>
   <si>
-    <t>2026-07-20 04:48:09 UTC</t>
+    <t>2026-07-20 04:59:23 UTC</t>
   </si>
   <si>
     <t>Branch</t>
@@ -1265,7 +1265,7 @@
     <t>Commit</t>
   </si>
   <si>
-    <t>f5c0ab7</t>
+    <t>2dd4e06</t>
   </si>
   <si>
     <t>Total</t>

</xml_diff>

<commit_message>
📊 Update reports — Build #48
</commit_message>
<xml_diff>
--- a/reports/appium/Excel/Automation_Test_Report.xlsx
+++ b/reports/appium/Excel/Automation_Test_Report.xlsx
@@ -1247,13 +1247,13 @@
     <t>Build Number</t>
   </si>
   <si>
-    <t>47</t>
+    <t>48</t>
   </si>
   <si>
     <t>Execution Date</t>
   </si>
   <si>
-    <t>2026-07-20 04:59:23 UTC</t>
+    <t>2026-07-20 05:11:04 UTC</t>
   </si>
   <si>
     <t>Branch</t>
@@ -1265,7 +1265,7 @@
     <t>Commit</t>
   </si>
   <si>
-    <t>2dd4e06</t>
+    <t>a601b64</t>
   </si>
   <si>
     <t>Total</t>

</xml_diff>

<commit_message>
📊 Update reports — Build #49
</commit_message>
<xml_diff>
--- a/reports/appium/Excel/Automation_Test_Report.xlsx
+++ b/reports/appium/Excel/Automation_Test_Report.xlsx
@@ -1247,13 +1247,13 @@
     <t>Build Number</t>
   </si>
   <si>
-    <t>48</t>
+    <t>49</t>
   </si>
   <si>
     <t>Execution Date</t>
   </si>
   <si>
-    <t>2026-07-20 05:11:04 UTC</t>
+    <t>2026-07-20 05:17:32 UTC</t>
   </si>
   <si>
     <t>Branch</t>
@@ -1265,7 +1265,7 @@
     <t>Commit</t>
   </si>
   <si>
-    <t>a601b64</t>
+    <t>4642e1d</t>
   </si>
   <si>
     <t>Total</t>

</xml_diff>

<commit_message>
📊 Update reports — Build #50
</commit_message>
<xml_diff>
--- a/reports/appium/Excel/Automation_Test_Report.xlsx
+++ b/reports/appium/Excel/Automation_Test_Report.xlsx
@@ -1247,13 +1247,13 @@
     <t>Build Number</t>
   </si>
   <si>
-    <t>49</t>
+    <t>50</t>
   </si>
   <si>
     <t>Execution Date</t>
   </si>
   <si>
-    <t>2026-07-20 05:17:32 UTC</t>
+    <t>2026-07-20 05:23:43 UTC</t>
   </si>
   <si>
     <t>Branch</t>
@@ -1265,7 +1265,7 @@
     <t>Commit</t>
   </si>
   <si>
-    <t>4642e1d</t>
+    <t>6ff8f77</t>
   </si>
   <si>
     <t>Total</t>

</xml_diff>

<commit_message>
📊 Update reports — Build #51
</commit_message>
<xml_diff>
--- a/reports/appium/Excel/Automation_Test_Report.xlsx
+++ b/reports/appium/Excel/Automation_Test_Report.xlsx
@@ -1247,13 +1247,13 @@
     <t>Build Number</t>
   </si>
   <si>
-    <t>50</t>
+    <t>51</t>
   </si>
   <si>
     <t>Execution Date</t>
   </si>
   <si>
-    <t>2026-07-20 05:23:43 UTC</t>
+    <t>2026-07-20 05:31:54 UTC</t>
   </si>
   <si>
     <t>Branch</t>
@@ -1265,7 +1265,7 @@
     <t>Commit</t>
   </si>
   <si>
-    <t>6ff8f77</t>
+    <t>521b99b</t>
   </si>
   <si>
     <t>Total</t>

</xml_diff>

<commit_message>
📊 Update reports — Build #52
</commit_message>
<xml_diff>
--- a/reports/appium/Excel/Automation_Test_Report.xlsx
+++ b/reports/appium/Excel/Automation_Test_Report.xlsx
@@ -1247,13 +1247,13 @@
     <t>Build Number</t>
   </si>
   <si>
-    <t>51</t>
+    <t>52</t>
   </si>
   <si>
     <t>Execution Date</t>
   </si>
   <si>
-    <t>2026-07-20 05:31:54 UTC</t>
+    <t>2026-07-20 05:38:08 UTC</t>
   </si>
   <si>
     <t>Branch</t>
@@ -1265,7 +1265,7 @@
     <t>Commit</t>
   </si>
   <si>
-    <t>521b99b</t>
+    <t>44e8e58</t>
   </si>
   <si>
     <t>Total</t>

</xml_diff>

<commit_message>
📊 Update reports — Build #53
</commit_message>
<xml_diff>
--- a/reports/appium/Excel/Automation_Test_Report.xlsx
+++ b/reports/appium/Excel/Automation_Test_Report.xlsx
@@ -1247,13 +1247,13 @@
     <t>Build Number</t>
   </si>
   <si>
-    <t>52</t>
+    <t>53</t>
   </si>
   <si>
     <t>Execution Date</t>
   </si>
   <si>
-    <t>2026-07-20 05:38:08 UTC</t>
+    <t>2026-07-20 05:49:54 UTC</t>
   </si>
   <si>
     <t>Branch</t>
@@ -1265,7 +1265,7 @@
     <t>Commit</t>
   </si>
   <si>
-    <t>44e8e58</t>
+    <t>d05746b</t>
   </si>
   <si>
     <t>Total</t>

</xml_diff>

<commit_message>
📊 Update reports — Build #54
</commit_message>
<xml_diff>
--- a/reports/appium/Excel/Automation_Test_Report.xlsx
+++ b/reports/appium/Excel/Automation_Test_Report.xlsx
@@ -1247,13 +1247,13 @@
     <t>Build Number</t>
   </si>
   <si>
-    <t>53</t>
+    <t>54</t>
   </si>
   <si>
     <t>Execution Date</t>
   </si>
   <si>
-    <t>2026-07-20 05:49:54 UTC</t>
+    <t>2026-07-20 06:05:56 UTC</t>
   </si>
   <si>
     <t>Branch</t>
@@ -1265,7 +1265,7 @@
     <t>Commit</t>
   </si>
   <si>
-    <t>d05746b</t>
+    <t>c2b056c</t>
   </si>
   <si>
     <t>Total</t>

</xml_diff>

<commit_message>
📊 Update reports — Build #55
</commit_message>
<xml_diff>
--- a/reports/appium/Excel/Automation_Test_Report.xlsx
+++ b/reports/appium/Excel/Automation_Test_Report.xlsx
@@ -1247,13 +1247,13 @@
     <t>Build Number</t>
   </si>
   <si>
-    <t>54</t>
+    <t>55</t>
   </si>
   <si>
     <t>Execution Date</t>
   </si>
   <si>
-    <t>2026-07-20 06:05:56 UTC</t>
+    <t>2026-07-20 06:13:22 UTC</t>
   </si>
   <si>
     <t>Branch</t>
@@ -1265,7 +1265,7 @@
     <t>Commit</t>
   </si>
   <si>
-    <t>c2b056c</t>
+    <t>6166361</t>
   </si>
   <si>
     <t>Total</t>

</xml_diff>

<commit_message>
📊 Update reports — Build #56
</commit_message>
<xml_diff>
--- a/reports/appium/Excel/Automation_Test_Report.xlsx
+++ b/reports/appium/Excel/Automation_Test_Report.xlsx
@@ -1247,13 +1247,13 @@
     <t>Build Number</t>
   </si>
   <si>
-    <t>55</t>
+    <t>56</t>
   </si>
   <si>
     <t>Execution Date</t>
   </si>
   <si>
-    <t>2026-07-20 06:13:22 UTC</t>
+    <t>2026-07-20 11:12:45 UTC</t>
   </si>
   <si>
     <t>Branch</t>
@@ -1265,7 +1265,7 @@
     <t>Commit</t>
   </si>
   <si>
-    <t>6166361</t>
+    <t>ea04ba1</t>
   </si>
   <si>
     <t>Total</t>

</xml_diff>

<commit_message>
📊 Update reports — Build #57
</commit_message>
<xml_diff>
--- a/reports/appium/Excel/Automation_Test_Report.xlsx
+++ b/reports/appium/Excel/Automation_Test_Report.xlsx
@@ -1247,13 +1247,13 @@
     <t>Build Number</t>
   </si>
   <si>
-    <t>56</t>
+    <t>57</t>
   </si>
   <si>
     <t>Execution Date</t>
   </si>
   <si>
-    <t>2026-07-20 11:12:45 UTC</t>
+    <t>2026-07-20 11:26:24 UTC</t>
   </si>
   <si>
     <t>Branch</t>
@@ -1265,7 +1265,7 @@
     <t>Commit</t>
   </si>
   <si>
-    <t>ea04ba1</t>
+    <t>444b861</t>
   </si>
   <si>
     <t>Total</t>

</xml_diff>

<commit_message>
📊 Update reports — Build #58
</commit_message>
<xml_diff>
--- a/reports/appium/Excel/Automation_Test_Report.xlsx
+++ b/reports/appium/Excel/Automation_Test_Report.xlsx
@@ -1247,13 +1247,13 @@
     <t>Build Number</t>
   </si>
   <si>
-    <t>57</t>
+    <t>58</t>
   </si>
   <si>
     <t>Execution Date</t>
   </si>
   <si>
-    <t>2026-07-20 11:26:24 UTC</t>
+    <t>2026-07-20 11:33:04 UTC</t>
   </si>
   <si>
     <t>Branch</t>
@@ -1265,7 +1265,7 @@
     <t>Commit</t>
   </si>
   <si>
-    <t>444b861</t>
+    <t>2507a7b</t>
   </si>
   <si>
     <t>Total</t>

</xml_diff>

<commit_message>
📊 Update reports — Build #59
</commit_message>
<xml_diff>
--- a/reports/appium/Excel/Automation_Test_Report.xlsx
+++ b/reports/appium/Excel/Automation_Test_Report.xlsx
@@ -1247,13 +1247,13 @@
     <t>Build Number</t>
   </si>
   <si>
-    <t>58</t>
+    <t>59</t>
   </si>
   <si>
     <t>Execution Date</t>
   </si>
   <si>
-    <t>2026-07-20 11:33:04 UTC</t>
+    <t>2026-07-20 15:13:39 UTC</t>
   </si>
   <si>
     <t>Branch</t>
@@ -1265,7 +1265,7 @@
     <t>Commit</t>
   </si>
   <si>
-    <t>2507a7b</t>
+    <t>8511c2b</t>
   </si>
   <si>
     <t>Total</t>

</xml_diff>

<commit_message>
📊 Update reports — Build #60
</commit_message>
<xml_diff>
--- a/reports/appium/Excel/Automation_Test_Report.xlsx
+++ b/reports/appium/Excel/Automation_Test_Report.xlsx
@@ -1247,13 +1247,13 @@
     <t>Build Number</t>
   </si>
   <si>
-    <t>59</t>
+    <t>60</t>
   </si>
   <si>
     <t>Execution Date</t>
   </si>
   <si>
-    <t>2026-07-20 15:13:39 UTC</t>
+    <t>2026-07-20 15:26:30 UTC</t>
   </si>
   <si>
     <t>Branch</t>
@@ -1265,7 +1265,7 @@
     <t>Commit</t>
   </si>
   <si>
-    <t>8511c2b</t>
+    <t>0291447</t>
   </si>
   <si>
     <t>Total</t>

</xml_diff>

<commit_message>
📊 Update reports — Build #61
</commit_message>
<xml_diff>
--- a/reports/appium/Excel/Automation_Test_Report.xlsx
+++ b/reports/appium/Excel/Automation_Test_Report.xlsx
@@ -1247,13 +1247,13 @@
     <t>Build Number</t>
   </si>
   <si>
-    <t>60</t>
+    <t>61</t>
   </si>
   <si>
     <t>Execution Date</t>
   </si>
   <si>
-    <t>2026-07-20 15:26:30 UTC</t>
+    <t>2026-07-21 10:04:43 UTC</t>
   </si>
   <si>
     <t>Branch</t>
@@ -1265,7 +1265,7 @@
     <t>Commit</t>
   </si>
   <si>
-    <t>0291447</t>
+    <t>00ba088</t>
   </si>
   <si>
     <t>Total</t>

</xml_diff>

<commit_message>
📊 Update reports — Build #62
</commit_message>
<xml_diff>
--- a/reports/appium/Excel/Automation_Test_Report.xlsx
+++ b/reports/appium/Excel/Automation_Test_Report.xlsx
@@ -1247,13 +1247,13 @@
     <t>Build Number</t>
   </si>
   <si>
-    <t>61</t>
+    <t>62</t>
   </si>
   <si>
     <t>Execution Date</t>
   </si>
   <si>
-    <t>2026-07-21 10:04:43 UTC</t>
+    <t>2026-07-21 10:32:58 UTC</t>
   </si>
   <si>
     <t>Branch</t>
@@ -1265,7 +1265,7 @@
     <t>Commit</t>
   </si>
   <si>
-    <t>00ba088</t>
+    <t>536fb94</t>
   </si>
   <si>
     <t>Total</t>

</xml_diff>

<commit_message>
📊 Update reports — Build #63
</commit_message>
<xml_diff>
--- a/reports/appium/Excel/Automation_Test_Report.xlsx
+++ b/reports/appium/Excel/Automation_Test_Report.xlsx
@@ -1247,13 +1247,13 @@
     <t>Build Number</t>
   </si>
   <si>
-    <t>62</t>
+    <t>63</t>
   </si>
   <si>
     <t>Execution Date</t>
   </si>
   <si>
-    <t>2026-07-21 10:32:58 UTC</t>
+    <t>2026-07-21 10:56:13 UTC</t>
   </si>
   <si>
     <t>Branch</t>
@@ -1265,7 +1265,7 @@
     <t>Commit</t>
   </si>
   <si>
-    <t>536fb94</t>
+    <t>9c8f524</t>
   </si>
   <si>
     <t>Total</t>

</xml_diff>

<commit_message>
📊 Update reports — Build #64
</commit_message>
<xml_diff>
--- a/reports/appium/Excel/Automation_Test_Report.xlsx
+++ b/reports/appium/Excel/Automation_Test_Report.xlsx
@@ -1247,13 +1247,13 @@
     <t>Build Number</t>
   </si>
   <si>
-    <t>63</t>
+    <t>64</t>
   </si>
   <si>
     <t>Execution Date</t>
   </si>
   <si>
-    <t>2026-07-21 10:56:13 UTC</t>
+    <t>2026-07-21 13:08:39 UTC</t>
   </si>
   <si>
     <t>Branch</t>
@@ -1265,7 +1265,7 @@
     <t>Commit</t>
   </si>
   <si>
-    <t>9c8f524</t>
+    <t>ed920c1</t>
   </si>
   <si>
     <t>Total</t>

</xml_diff>

<commit_message>
📊 Update reports — Build #65
</commit_message>
<xml_diff>
--- a/reports/appium/Excel/Automation_Test_Report.xlsx
+++ b/reports/appium/Excel/Automation_Test_Report.xlsx
@@ -1247,13 +1247,13 @@
     <t>Build Number</t>
   </si>
   <si>
-    <t>64</t>
+    <t>65</t>
   </si>
   <si>
     <t>Execution Date</t>
   </si>
   <si>
-    <t>2026-07-21 13:08:39 UTC</t>
+    <t>2026-07-21 13:43:10 UTC</t>
   </si>
   <si>
     <t>Branch</t>
@@ -1265,7 +1265,7 @@
     <t>Commit</t>
   </si>
   <si>
-    <t>ed920c1</t>
+    <t>f0162ef</t>
   </si>
   <si>
     <t>Total</t>

</xml_diff>

<commit_message>
📊 Update reports — Build #66
</commit_message>
<xml_diff>
--- a/reports/appium/Excel/Automation_Test_Report.xlsx
+++ b/reports/appium/Excel/Automation_Test_Report.xlsx
@@ -1247,13 +1247,13 @@
     <t>Build Number</t>
   </si>
   <si>
-    <t>65</t>
+    <t>66</t>
   </si>
   <si>
     <t>Execution Date</t>
   </si>
   <si>
-    <t>2026-07-21 13:43:10 UTC</t>
+    <t>2026-07-21 13:54:01 UTC</t>
   </si>
   <si>
     <t>Branch</t>
@@ -1265,7 +1265,7 @@
     <t>Commit</t>
   </si>
   <si>
-    <t>f0162ef</t>
+    <t>c20f7b4</t>
   </si>
   <si>
     <t>Total</t>

</xml_diff>

<commit_message>
📊 Update reports — Build #67
</commit_message>
<xml_diff>
--- a/reports/appium/Excel/Automation_Test_Report.xlsx
+++ b/reports/appium/Excel/Automation_Test_Report.xlsx
@@ -1247,13 +1247,13 @@
     <t>Build Number</t>
   </si>
   <si>
-    <t>66</t>
+    <t>67</t>
   </si>
   <si>
     <t>Execution Date</t>
   </si>
   <si>
-    <t>2026-07-21 13:54:01 UTC</t>
+    <t>2026-07-21 14:13:19 UTC</t>
   </si>
   <si>
     <t>Branch</t>
@@ -1265,7 +1265,7 @@
     <t>Commit</t>
   </si>
   <si>
-    <t>c20f7b4</t>
+    <t>77d93ce</t>
   </si>
   <si>
     <t>Total</t>

</xml_diff>

<commit_message>
📊 Update reports — Build #68
</commit_message>
<xml_diff>
--- a/reports/appium/Excel/Automation_Test_Report.xlsx
+++ b/reports/appium/Excel/Automation_Test_Report.xlsx
@@ -1247,13 +1247,13 @@
     <t>Build Number</t>
   </si>
   <si>
-    <t>67</t>
+    <t>68</t>
   </si>
   <si>
     <t>Execution Date</t>
   </si>
   <si>
-    <t>2026-07-21 14:13:19 UTC</t>
+    <t>2026-07-21 14:22:49 UTC</t>
   </si>
   <si>
     <t>Branch</t>
@@ -1265,7 +1265,7 @@
     <t>Commit</t>
   </si>
   <si>
-    <t>77d93ce</t>
+    <t>14f8400</t>
   </si>
   <si>
     <t>Total</t>

</xml_diff>

<commit_message>
📊 Update reports — Build #69
</commit_message>
<xml_diff>
--- a/reports/appium/Excel/Automation_Test_Report.xlsx
+++ b/reports/appium/Excel/Automation_Test_Report.xlsx
@@ -1247,13 +1247,13 @@
     <t>Build Number</t>
   </si>
   <si>
-    <t>68</t>
+    <t>69</t>
   </si>
   <si>
     <t>Execution Date</t>
   </si>
   <si>
-    <t>2026-07-21 14:22:49 UTC</t>
+    <t>2026-07-21 14:37:15 UTC</t>
   </si>
   <si>
     <t>Branch</t>
@@ -1265,7 +1265,7 @@
     <t>Commit</t>
   </si>
   <si>
-    <t>14f8400</t>
+    <t>087f127</t>
   </si>
   <si>
     <t>Total</t>

</xml_diff>

<commit_message>
📊 Update reports — Build #70
</commit_message>
<xml_diff>
--- a/reports/appium/Excel/Automation_Test_Report.xlsx
+++ b/reports/appium/Excel/Automation_Test_Report.xlsx
@@ -1247,13 +1247,13 @@
     <t>Build Number</t>
   </si>
   <si>
-    <t>69</t>
+    <t>70</t>
   </si>
   <si>
     <t>Execution Date</t>
   </si>
   <si>
-    <t>2026-07-21 14:37:15 UTC</t>
+    <t>2026-07-21 15:10:01 UTC</t>
   </si>
   <si>
     <t>Branch</t>
@@ -1265,7 +1265,7 @@
     <t>Commit</t>
   </si>
   <si>
-    <t>087f127</t>
+    <t>6958884</t>
   </si>
   <si>
     <t>Total</t>

</xml_diff>

<commit_message>
📊 Update reports — Build #71
</commit_message>
<xml_diff>
--- a/reports/appium/Excel/Automation_Test_Report.xlsx
+++ b/reports/appium/Excel/Automation_Test_Report.xlsx
@@ -1247,13 +1247,13 @@
     <t>Build Number</t>
   </si>
   <si>
-    <t>70</t>
+    <t>71</t>
   </si>
   <si>
     <t>Execution Date</t>
   </si>
   <si>
-    <t>2026-07-21 15:10:01 UTC</t>
+    <t>2026-07-22 02:02:21 UTC</t>
   </si>
   <si>
     <t>Branch</t>
@@ -1265,7 +1265,7 @@
     <t>Commit</t>
   </si>
   <si>
-    <t>6958884</t>
+    <t>2d71144</t>
   </si>
   <si>
     <t>Total</t>

</xml_diff>

<commit_message>
📊 Update reports — Build #72
</commit_message>
<xml_diff>
--- a/reports/appium/Excel/Automation_Test_Report.xlsx
+++ b/reports/appium/Excel/Automation_Test_Report.xlsx
@@ -1247,13 +1247,13 @@
     <t>Build Number</t>
   </si>
   <si>
-    <t>71</t>
+    <t>72</t>
   </si>
   <si>
     <t>Execution Date</t>
   </si>
   <si>
-    <t>2026-07-22 02:02:21 UTC</t>
+    <t>2026-07-22 02:47:22 UTC</t>
   </si>
   <si>
     <t>Branch</t>
@@ -1265,7 +1265,7 @@
     <t>Commit</t>
   </si>
   <si>
-    <t>2d71144</t>
+    <t>a96e094</t>
   </si>
   <si>
     <t>Total</t>

</xml_diff>

<commit_message>
📊 Update reports — Build #73
</commit_message>
<xml_diff>
--- a/reports/appium/Excel/Automation_Test_Report.xlsx
+++ b/reports/appium/Excel/Automation_Test_Report.xlsx
@@ -1247,13 +1247,13 @@
     <t>Build Number</t>
   </si>
   <si>
-    <t>72</t>
+    <t>73</t>
   </si>
   <si>
     <t>Execution Date</t>
   </si>
   <si>
-    <t>2026-07-22 02:47:22 UTC</t>
+    <t>2026-07-22 02:54:06 UTC</t>
   </si>
   <si>
     <t>Branch</t>
@@ -1265,7 +1265,7 @@
     <t>Commit</t>
   </si>
   <si>
-    <t>a96e094</t>
+    <t>adc634e</t>
   </si>
   <si>
     <t>Total</t>

</xml_diff>

<commit_message>
📊 Update reports — Build #78
</commit_message>
<xml_diff>
--- a/reports/appium/Excel/Automation_Test_Report.xlsx
+++ b/reports/appium/Excel/Automation_Test_Report.xlsx
@@ -1247,13 +1247,13 @@
     <t>Build Number</t>
   </si>
   <si>
-    <t>77</t>
+    <t>78</t>
   </si>
   <si>
     <t>Execution Date</t>
   </si>
   <si>
-    <t>2026-07-22 03:38:07 UTC</t>
+    <t>2026-07-22 03:44:10 UTC</t>
   </si>
   <si>
     <t>Branch</t>
@@ -1265,7 +1265,7 @@
     <t>Commit</t>
   </si>
   <si>
-    <t>b0c83f8</t>
+    <t>6a5de8e</t>
   </si>
   <si>
     <t>Total</t>

</xml_diff>

<commit_message>
📊 Update reports — Build #81
</commit_message>
<xml_diff>
--- a/reports/appium/Excel/Automation_Test_Report.xlsx
+++ b/reports/appium/Excel/Automation_Test_Report.xlsx
@@ -1247,13 +1247,13 @@
     <t>Build Number</t>
   </si>
   <si>
-    <t>80</t>
+    <t>81</t>
   </si>
   <si>
     <t>Execution Date</t>
   </si>
   <si>
-    <t>2026-07-22 04:11:53 UTC</t>
+    <t>2026-07-22 04:18:20 UTC</t>
   </si>
   <si>
     <t>Branch</t>
@@ -1265,7 +1265,7 @@
     <t>Commit</t>
   </si>
   <si>
-    <t>e4fdde1</t>
+    <t>49466e1</t>
   </si>
   <si>
     <t>Total</t>

</xml_diff>

<commit_message>
📊 Update reports — Build #82
</commit_message>
<xml_diff>
--- a/reports/appium/Excel/Automation_Test_Report.xlsx
+++ b/reports/appium/Excel/Automation_Test_Report.xlsx
@@ -1247,13 +1247,13 @@
     <t>Build Number</t>
   </si>
   <si>
-    <t>81</t>
+    <t>82</t>
   </si>
   <si>
     <t>Execution Date</t>
   </si>
   <si>
-    <t>2026-07-23 08:24:06 UTC</t>
+    <t>2026-07-30 09:23:08 UTC</t>
   </si>
   <si>
     <t>Branch</t>
@@ -1265,7 +1265,7 @@
     <t>Commit</t>
   </si>
   <si>
-    <t>49466e1</t>
+    <t>c1ecc81</t>
   </si>
   <si>
     <t>Total</t>

</xml_diff>